<commit_message>
Replace the chair of session 38 with a VMTW standby
Dr. Ratnesh Litoriya cannot attend. V. D. V. Nagalakshmi, a VMTW standby volunteer
with no paper in the programme, chairs session 38, Clinical Intelligence and Healthcare
Digital Twins, Tuesday 10:00-11:12, with the Meet link they supplied. The session now
has a link. The session 38 chair sheet is regenerated to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/programme/chair-sheets/S38.xlsx
+++ b/programme/chair-sheets/S38.xlsx
@@ -46,7 +46,7 @@
     <t xml:space="preserve">Session chair</t>
   </si>
   <si>
-    <t xml:space="preserve">Dr. Ratnesh Litoriya</t>
+    <t xml:space="preserve">V. D. V. Nagalakshmi</t>
   </si>
   <si>
     <t xml:space="preserve">Co-chair</t>
@@ -58,7 +58,7 @@
     <t xml:space="preserve">Joining link</t>
   </si>
   <si>
-    <t xml:space="preserve">to be confirmed</t>
+    <t xml:space="preserve">https://meet.google.com/vgs-ruvf-jtt</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>

</xml_diff>